<commit_message>
Recalibrate solar supply curve
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-analysis\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCE1167F-B04F-40E6-B755-712DE2FE0ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BE2E95-F00F-425C-AE89-A258C20FEB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="4545" yWindow="3765" windowWidth="21600" windowHeight="12645" activeTab="3" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="101">
   <si>
     <t xml:space="preserve">Source: </t>
   </si>
@@ -338,6 +338,9 @@
   </si>
   <si>
     <t>2 projects; shares gas-turbine supply chain</t>
+  </si>
+  <si>
+    <t>Update 2026-09-24 (solar PV): Share of Cost Effective Capacity Built in a Single Year for solar PV set to 0.5 in all years (deployed CSV had carried 0.75 since the 2026-09-11 calibration while this workbook still showed 1.0; both now 0.5). Rationale: at 0.75 the economic channel added 38-45 GW/yr of solar in 2027-2029 on top of the mandated pipeline (52/47/42 GW/yr total; 2030 capacity 360 GW) against ICF's forecast of 34-39 GW/yr and 2025's record ~30 GW, with solar curtailment of 53-57 TWh/yr. At 0.5, additions are 41/32/28 GW/yr and 2030 capacity 313 GW, between ReEDS StdScen24 Mid (~330) and Rhodium TS2026 Mid (262). Same 'reflect real-world builds' logic as the onshore wind values. Decision: Megan, 2026-09-24. A post-2030 dip in economic solar (profitability saturation via the CSC saturation parameter) is unaffected by this share.</t>
   </si>
 </sst>
 </file>
@@ -484,7 +487,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>About!$C$25:$C$125</c:f>
+              <c:f>About!$C$27:$C$127</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
@@ -796,7 +799,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>About!$B$25:$B$125</c:f>
+              <c:f>About!$B$27:$B$127</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
@@ -1862,13 +1865,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>484003</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>184356</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>5052459</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>171656</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2194,7 +2197,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
-  <dimension ref="A1:C157"/>
+  <dimension ref="A1:C159"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
@@ -2250,1257 +2253,1240 @@
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17">
-        <v>0.6</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B19">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B20">
-        <v>30000</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>37</v>
       </c>
-      <c r="B21">
+      <c r="B23">
         <v>4.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B24">
-        <f>(1-EXP(-((C24/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
-        <v>0</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B25">
-        <f t="shared" ref="B25:B88" si="0">(1-EXP(-((C25/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
-        <v>4.286648162477036E-6</v>
-      </c>
-      <c r="C25">
-        <v>500</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26">
-        <f t="shared" si="0"/>
-        <v>3.4290612860687911E-5</v>
+        <f>(1-EXP(-((C26/$B$22-($B$21-0.5))/$B$19)^$B$20))*$B$18</f>
+        <v>0</v>
       </c>
       <c r="C26">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27">
-        <f t="shared" si="0"/>
-        <v>1.1570725740235322E-4</v>
+        <f t="shared" ref="B27:B90" si="0">(1-EXP(-((C27/$B$22-($B$21-0.5))/$B$19)^$B$20))*$B$18</f>
+        <v>4.286648162477036E-6</v>
       </c>
       <c r="C27">
-        <f>C26+500</f>
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>2.7416034086391594E-4</v>
+        <v>3.4290612860687911E-5</v>
       </c>
       <c r="C28">
-        <f t="shared" ref="C28:C91" si="1">C27+500</f>
-        <v>2000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>5.3511960071055413E-4</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="C29">
-        <f t="shared" si="1"/>
-        <v>2500</v>
+        <f>C28+500</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>9.2378588268478008E-4</v>
+        <v>2.7416034086391594E-4</v>
       </c>
       <c r="C30">
-        <f t="shared" si="1"/>
-        <v>3000</v>
+        <f t="shared" ref="C30:C93" si="1">C29+500</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>1.4649445766562463E-3</v>
+        <v>5.3511960071055413E-4</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
-        <v>3500</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32">
         <f t="shared" si="0"/>
-        <v>2.1827885823227922E-3</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="C32">
         <f t="shared" si="1"/>
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>3.1007125989183093E-3</v>
+        <v>1.4649445766562463E-3</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
-        <v>4500</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>4.2410811978808027E-3</v>
+        <v>2.1827885823227922E-3</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
-        <v>5000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <f t="shared" si="0"/>
-        <v>5.6249738820245872E-3</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="C35">
         <f t="shared" si="1"/>
-        <v>5500</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>7.2719111397427484E-3</v>
+        <v>4.2410811978808027E-3</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
-        <v>6000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>9.1995663437769003E-3</v>
+        <v>5.6249738820245872E-3</v>
       </c>
       <c r="C37">
         <f t="shared" si="1"/>
-        <v>6500</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>1.1423469191788382E-2</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="C38">
         <f t="shared" si="1"/>
-        <v>7000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>1.3956707206263963E-2</v>
+        <v>9.1995663437769003E-3</v>
       </c>
       <c r="C39">
         <f t="shared" si="1"/>
-        <v>7500</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>1.6809632565965439E-2</v>
+        <v>1.1423469191788382E-2</v>
       </c>
       <c r="C40">
         <f t="shared" si="1"/>
-        <v>8000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>1.9989582188770449E-2</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
-        <v>8500</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>2.3500619483080909E-2</v>
+        <v>1.6809632565965439E-2</v>
       </c>
       <c r="C42">
         <f t="shared" si="1"/>
-        <v>9000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>2.7343306488591249E-2</v>
+        <v>1.9989582188770449E-2</v>
       </c>
       <c r="C43">
         <f t="shared" si="1"/>
-        <v>9500</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>3.1514515195616613E-2</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="C44">
         <f t="shared" si="1"/>
-        <v>10000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>3.6007286628151627E-2</v>
+        <v>2.7343306488591249E-2</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
-        <v>10500</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>4.0810745768913415E-2</v>
+        <v>3.1514515195616613E-2</v>
       </c>
       <c r="C46">
         <f t="shared" si="1"/>
-        <v>11000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>4.5910079573753593E-2</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="C47">
         <f t="shared" si="1"/>
-        <v>11500</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>5.1286584158818753E-2</v>
+        <v>4.0810745768913415E-2</v>
       </c>
       <c r="C48">
         <f t="shared" si="1"/>
-        <v>12000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>5.6917785751641151E-2</v>
+        <v>4.5910079573753593E-2</v>
       </c>
       <c r="C49">
         <f t="shared" si="1"/>
-        <v>12500</v>
+        <v>11500</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>6.2777638197790697E-2</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="C50">
         <f t="shared" si="1"/>
-        <v>13000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>6.8836797745699688E-2</v>
+        <v>5.6917785751641151E-2</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
-        <v>13500</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>7.506297354898428E-2</v>
+        <v>6.2777638197790697E-2</v>
       </c>
       <c r="C52">
         <f t="shared" si="1"/>
-        <v>14000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>8.142134989988481E-2</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="C53">
         <f t="shared" si="1"/>
-        <v>14500</v>
+        <v>13500</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>8.787507372604586E-2</v>
+        <v>7.506297354898428E-2</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
-        <v>15000</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>9.438579844442066E-2</v>
+        <v>8.142134989988481E-2</v>
       </c>
       <c r="C55">
         <f t="shared" si="1"/>
-        <v>15500</v>
+        <v>14500</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>0.10091427297723279</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
-        <v>16000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>0.10742096270522571</v>
+        <v>9.438579844442066E-2</v>
       </c>
       <c r="C57">
         <f t="shared" si="1"/>
-        <v>16500</v>
+        <v>15500</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>0.11386668746965854</v>
+        <v>0.10091427297723279</v>
       </c>
       <c r="C58">
         <f t="shared" si="1"/>
-        <v>17000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>0.12021326053442474</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="C59">
         <f t="shared" si="1"/>
-        <v>17500</v>
+        <v>16500</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>0.12642411176571153</v>
+        <v>0.11386668746965854</v>
       </c>
       <c r="C60">
         <f t="shared" si="1"/>
-        <v>18000</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>0.1324648782399141</v>
+        <v>0.12021326053442474</v>
       </c>
       <c r="C61">
         <f t="shared" si="1"/>
-        <v>18500</v>
+        <v>17500</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>0.1383039460856948</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="C62">
         <f t="shared" si="1"/>
-        <v>19000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>0.1439129286073208</v>
+        <v>0.1324648782399141</v>
       </c>
       <c r="C63">
         <f t="shared" si="1"/>
-        <v>19500</v>
+        <v>18500</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>0.14926706759510625</v>
+        <v>0.1383039460856948</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
-        <v>20000</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>0.15434554714316789</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
-        <v>20500</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>0.1591317121715517</v>
+        <v>0.14926706759510625</v>
       </c>
       <c r="C66">
         <f t="shared" si="1"/>
-        <v>21000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>0.16361318706836692</v>
+        <v>0.15434554714316789</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
-        <v>21500</v>
+        <v>20500</v>
       </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
         <f t="shared" si="0"/>
-        <v>0.16778189328550838</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="C68">
         <f t="shared" si="1"/>
-        <v>22000</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
         <f t="shared" si="0"/>
-        <v>0.17163396818253152</v>
+        <v>0.16361318706836692</v>
       </c>
       <c r="C69">
         <f t="shared" si="1"/>
-        <v>22500</v>
+        <v>21500</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
         <f t="shared" si="0"/>
-        <v>0.17516959075587743</v>
+        <v>0.16778189328550838</v>
       </c>
       <c r="C70">
         <f t="shared" si="1"/>
-        <v>23000</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
         <f t="shared" si="0"/>
-        <v>0.17839272295802988</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="C71">
         <f t="shared" si="1"/>
-        <v>23500</v>
+        <v>22500</v>
       </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
         <f t="shared" si="0"/>
-        <v>0.18131077796047496</v>
+        <v>0.17516959075587743</v>
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
         <f t="shared" si="0"/>
-        <v>0.18393422882553601</v>
+        <v>0.17839272295802988</v>
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
-        <v>24500</v>
+        <v>23500</v>
       </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
         <f t="shared" si="0"/>
-        <v>0.18627617253555084</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
-        <v>25000</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
         <f t="shared" si="0"/>
-        <v>0.18835186512938695</v>
+        <v>0.18393422882553601</v>
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
-        <v>25500</v>
+        <v>24500</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76">
         <f t="shared" si="0"/>
-        <v>0.19017824380056211</v>
+        <v>0.18627617253555084</v>
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
-        <v>26000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77">
         <f t="shared" si="0"/>
-        <v>0.19177345124178691</v>
+        <v>0.18835186512938695</v>
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
-        <v>26500</v>
+        <v>25500</v>
       </c>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B78">
         <f t="shared" si="0"/>
-        <v>0.1931563763376668</v>
+        <v>0.19017824380056211</v>
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
-        <v>27000</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79">
         <f t="shared" si="0"/>
-        <v>0.19434622360232301</v>
+        <v>0.19177345124178691</v>
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
-        <v>27500</v>
+        <v>26500</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80">
         <f t="shared" si="0"/>
-        <v>0.19536212164822028</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
-        <v>28000</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81">
         <f t="shared" si="0"/>
-        <v>0.19622277858911699</v>
+        <v>0.19434622360232301</v>
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
-        <v>28500</v>
+        <v>27500</v>
       </c>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82">
         <f t="shared" si="0"/>
-        <v>0.19694618976330103</v>
+        <v>0.19536212164822028</v>
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
-        <v>29000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83">
         <f t="shared" si="0"/>
-        <v>0.19754940065027685</v>
+        <v>0.19622277858911699</v>
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
-        <v>29500</v>
+        <v>28500</v>
       </c>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84">
         <f t="shared" si="0"/>
-        <v>0.19804832547095644</v>
+        <v>0.19694618976330103</v>
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
-        <v>30000</v>
+        <v>29000</v>
       </c>
     </row>
     <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85">
         <f t="shared" si="0"/>
-        <v>0.19845761981600954</v>
+        <v>0.19754940065027685</v>
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
-        <v>30500</v>
+        <v>29500</v>
       </c>
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86">
         <f t="shared" si="0"/>
-        <v>0.19879060382342864</v>
+        <v>0.19804832547095644</v>
       </c>
       <c r="C86">
         <f t="shared" si="1"/>
-        <v>31000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87">
         <f t="shared" si="0"/>
-        <v>0.19905923098155251</v>
+        <v>0.19845761981600954</v>
       </c>
       <c r="C87">
         <f t="shared" si="1"/>
-        <v>31500</v>
+        <v>30500</v>
       </c>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88">
         <f t="shared" si="0"/>
-        <v>0.19927409659660289</v>
+        <v>0.19879060382342864</v>
       </c>
       <c r="C88">
         <f t="shared" si="1"/>
-        <v>32000</v>
+        <v>31000</v>
       </c>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89">
-        <f t="shared" ref="B89:B125" si="2">(1-EXP(-((C89/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
-        <v>0.19944447933595111</v>
+        <f t="shared" si="0"/>
+        <v>0.19905923098155251</v>
       </c>
       <c r="C89">
         <f t="shared" si="1"/>
-        <v>32500</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90">
-        <f t="shared" si="2"/>
-        <v>0.19957840901739385</v>
+        <f t="shared" si="0"/>
+        <v>0.19927409659660289</v>
       </c>
       <c r="C90">
         <f t="shared" si="1"/>
-        <v>33000</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B91">
-        <f t="shared" si="2"/>
-        <v>0.19968275391843365</v>
+        <f t="shared" ref="B91:B127" si="2">(1-EXP(-((C91/$B$22-($B$21-0.5))/$B$19)^$B$20))*$B$18</f>
+        <v>0.19944447933595111</v>
       </c>
       <c r="C91">
         <f t="shared" si="1"/>
-        <v>33500</v>
+        <v>32500</v>
       </c>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92">
         <f t="shared" si="2"/>
-        <v>0.19976332127118276</v>
+        <v>0.19957840901739385</v>
       </c>
       <c r="C92">
-        <f t="shared" ref="C92:C125" si="3">C91+500</f>
-        <v>34000</v>
+        <f t="shared" si="1"/>
+        <v>33000</v>
       </c>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93">
         <f t="shared" si="2"/>
-        <v>0.19982496522253218</v>
+        <v>0.19968275391843365</v>
       </c>
       <c r="C93">
-        <f t="shared" si="3"/>
-        <v>34500</v>
+        <f t="shared" si="1"/>
+        <v>33500</v>
       </c>
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B94">
         <f t="shared" si="2"/>
-        <v>0.19987169730697774</v>
+        <v>0.19976332127118276</v>
       </c>
       <c r="C94">
-        <f t="shared" si="3"/>
-        <v>35000</v>
+        <f t="shared" ref="C94:C127" si="3">C93+500</f>
+        <v>34000</v>
       </c>
     </row>
     <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95">
         <f t="shared" si="2"/>
-        <v>0.19990679533419684</v>
+        <v>0.19982496522253218</v>
       </c>
       <c r="C95">
         <f t="shared" si="3"/>
-        <v>35500</v>
+        <v>34500</v>
       </c>
     </row>
     <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96">
         <f t="shared" si="2"/>
-        <v>0.1999329074744195</v>
+        <v>0.19987169730697774</v>
       </c>
       <c r="C96">
         <f t="shared" si="3"/>
-        <v>36000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B97">
         <f t="shared" si="2"/>
-        <v>0.19995214918026516</v>
+        <v>0.19990679533419684</v>
       </c>
       <c r="C97">
         <f t="shared" si="3"/>
-        <v>36500</v>
+        <v>35500</v>
       </c>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B98">
         <f t="shared" si="2"/>
-        <v>0.19996619137347427</v>
+        <v>0.1999329074744195</v>
       </c>
       <c r="C98">
         <f t="shared" si="3"/>
-        <v>37000</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="99" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B99">
         <f t="shared" si="2"/>
-        <v>0.19997633902006273</v>
+        <v>0.19995214918026516</v>
       </c>
       <c r="C99">
         <f t="shared" si="3"/>
-        <v>37500</v>
+        <v>36500</v>
       </c>
     </row>
     <row r="100" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B100">
         <f t="shared" si="2"/>
-        <v>0.19998359980055544</v>
+        <v>0.19996619137347427</v>
       </c>
       <c r="C100">
         <f t="shared" si="3"/>
-        <v>38000</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="101" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B101">
         <f t="shared" si="2"/>
-        <v>0.19998874304618811</v>
+        <v>0.19997633902006273</v>
       </c>
       <c r="C101">
         <f t="shared" si="3"/>
-        <v>38500</v>
+        <v>37500</v>
       </c>
     </row>
     <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B102">
         <f t="shared" si="2"/>
-        <v>0.19999234945911523</v>
+        <v>0.19998359980055544</v>
       </c>
       <c r="C102">
         <f t="shared" si="3"/>
-        <v>39000</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="103" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B103">
         <f t="shared" si="2"/>
-        <v>0.19999485237326678</v>
+        <v>0.19998874304618811</v>
       </c>
       <c r="C103">
         <f t="shared" si="3"/>
-        <v>39500</v>
+        <v>38500</v>
       </c>
     </row>
     <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B104">
         <f t="shared" si="2"/>
-        <v>0.1999965714557792</v>
+        <v>0.19999234945911523</v>
       </c>
       <c r="C104">
         <f t="shared" si="3"/>
-        <v>40000</v>
+        <v>39000</v>
       </c>
     </row>
     <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B105">
         <f t="shared" si="2"/>
-        <v>0.19999773981279137</v>
+        <v>0.19999485237326678</v>
       </c>
       <c r="C105">
         <f t="shared" si="3"/>
-        <v>40500</v>
+        <v>39500</v>
       </c>
     </row>
     <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B106">
         <f t="shared" si="2"/>
-        <v>0.19999852546471561</v>
+        <v>0.1999965714557792</v>
       </c>
       <c r="C106">
         <f t="shared" si="3"/>
-        <v>41000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="107" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B107">
         <f t="shared" si="2"/>
-        <v>0.19999904811129313</v>
+        <v>0.19999773981279137</v>
       </c>
       <c r="C107">
         <f t="shared" si="3"/>
-        <v>41500</v>
+        <v>40500</v>
       </c>
     </row>
     <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B108">
         <f t="shared" si="2"/>
-        <v>0.19999939203080119</v>
+        <v>0.19999852546471561</v>
       </c>
       <c r="C108">
         <f t="shared" si="3"/>
-        <v>42000</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="109" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B109">
         <f t="shared" si="2"/>
-        <v>0.19999961586354192</v>
+        <v>0.19999904811129313</v>
       </c>
       <c r="C109">
         <f t="shared" si="3"/>
-        <v>42500</v>
+        <v>41500</v>
       </c>
     </row>
     <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B110">
         <f t="shared" si="2"/>
-        <v>0.19999975992763294</v>
+        <v>0.19999939203080119</v>
       </c>
       <c r="C110">
         <f t="shared" si="3"/>
-        <v>43000</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B111">
         <f t="shared" si="2"/>
-        <v>0.19999985161306397</v>
+        <v>0.19999961586354192</v>
       </c>
       <c r="C111">
         <f t="shared" si="3"/>
-        <v>43500</v>
+        <v>42500</v>
       </c>
     </row>
     <row r="112" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B112">
         <f t="shared" si="2"/>
-        <v>0.19999990930357772</v>
+        <v>0.19999975992763294</v>
       </c>
       <c r="C112">
         <f t="shared" si="3"/>
-        <v>44000</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113">
         <f t="shared" si="2"/>
-        <v>0.19999994518873965</v>
+        <v>0.19999985161306397</v>
       </c>
       <c r="C113">
         <f t="shared" si="3"/>
-        <v>44500</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+        <v>43500</v>
+      </c>
+    </row>
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114">
         <f t="shared" si="2"/>
-        <v>0.19999996725245739</v>
+        <v>0.19999990930357772</v>
       </c>
       <c r="C114">
         <f t="shared" si="3"/>
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115">
         <f t="shared" si="2"/>
-        <v>0.19999998065979441</v>
+        <v>0.19999994518873965</v>
       </c>
       <c r="C115">
         <f t="shared" si="3"/>
-        <v>45500</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116">
         <f t="shared" si="2"/>
-        <v>0.19999998871085503</v>
+        <v>0.19999996725245739</v>
       </c>
       <c r="C116">
         <f t="shared" si="3"/>
-        <v>46000</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B117">
         <f t="shared" si="2"/>
-        <v>0.19999999348787459</v>
+        <v>0.19999998065979441</v>
       </c>
       <c r="C117">
         <f t="shared" si="3"/>
-        <v>46500</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45500</v>
+      </c>
+    </row>
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B118">
         <f t="shared" si="2"/>
-        <v>0.19999999628815057</v>
+        <v>0.19999998871085503</v>
       </c>
       <c r="C118">
         <f t="shared" si="3"/>
-        <v>47000</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119">
         <f t="shared" si="2"/>
-        <v>0.19999999790970302</v>
+        <v>0.19999999348787459</v>
       </c>
       <c r="C119">
         <f t="shared" si="3"/>
-        <v>47500</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+        <v>46500</v>
+      </c>
+    </row>
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120">
         <f t="shared" si="2"/>
-        <v>0.19999999883716038</v>
+        <v>0.19999999628815057</v>
       </c>
       <c r="C120">
         <f t="shared" si="3"/>
-        <v>48000</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121">
         <f t="shared" si="2"/>
-        <v>0.19999999936104543</v>
+        <v>0.19999999790970302</v>
       </c>
       <c r="C121">
         <f t="shared" si="3"/>
-        <v>48500</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+        <v>47500</v>
+      </c>
+    </row>
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122">
         <f t="shared" si="2"/>
-        <v>0.19999999965326104</v>
+        <v>0.19999999883716038</v>
       </c>
       <c r="C122">
         <f t="shared" si="3"/>
-        <v>49000</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123">
         <f t="shared" si="2"/>
-        <v>0.19999999981419306</v>
+        <v>0.19999999936104543</v>
       </c>
       <c r="C123">
         <f t="shared" si="3"/>
-        <v>49500</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+        <v>48500</v>
+      </c>
+    </row>
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124">
         <f t="shared" si="2"/>
-        <v>0.19999999990169129</v>
+        <v>0.19999999965326104</v>
       </c>
       <c r="C124">
         <f t="shared" si="3"/>
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+        <v>49000</v>
+      </c>
+    </row>
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B125">
         <f t="shared" si="2"/>
-        <v>0.19999999994865042</v>
+        <v>0.19999999981419306</v>
       </c>
       <c r="C125">
         <f t="shared" si="3"/>
+        <v>49500</v>
+      </c>
+    </row>
+    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B126">
+        <f t="shared" si="2"/>
+        <v>0.19999999990169129</v>
+      </c>
+      <c r="C126">
+        <f t="shared" si="3"/>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B127">
+        <f t="shared" si="2"/>
+        <v>0.19999999994865042</v>
+      </c>
+      <c r="C127">
+        <f t="shared" si="3"/>
         <v>50500</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>77</v>
-      </c>
-      <c r="B133" t="s">
-        <v>78</v>
-      </c>
-      <c r="C133" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>48</v>
-      </c>
-      <c r="B134">
-        <v>1300</v>
-      </c>
-      <c r="C134" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>49</v>
-      </c>
-      <c r="B135">
-        <v>600</v>
+        <v>77</v>
+      </c>
+      <c r="B135" t="s">
+        <v>78</v>
       </c>
       <c r="C135" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B136">
-        <v>10000</v>
+        <v>1300</v>
       </c>
       <c r="C136" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B137">
-        <v>2200</v>
+        <v>600</v>
       </c>
       <c r="C137" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B138">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="C138" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B139">
-        <v>15000</v>
+        <v>2200</v>
       </c>
       <c r="C139" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B140">
-        <v>30000</v>
+        <v>500</v>
       </c>
       <c r="C140" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B141">
-        <v>400</v>
+        <v>15000</v>
       </c>
       <c r="C141" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B142">
-        <v>500</v>
+        <v>30000</v>
       </c>
       <c r="C142" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B143">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="C143" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B144">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C144" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B145">
-        <v>5000</v>
+        <v>150</v>
       </c>
       <c r="C145" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B146">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="C146" t="s">
         <v>89</v>
@@ -3508,21 +3494,21 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B147">
-        <v>2400</v>
+        <v>5000</v>
       </c>
       <c r="C147" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B148">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C148" t="s">
         <v>89</v>
@@ -3530,100 +3516,122 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B149">
-        <v>200</v>
+        <v>2400</v>
       </c>
       <c r="C149" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B150">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C150" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B151">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="C151" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B152">
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="C152" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B153">
         <v>1000</v>
       </c>
       <c r="C153" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B154">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="C154" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B155">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="C155" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B156">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="C156" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
+        <v>69</v>
+      </c>
+      <c r="B157">
+        <v>1200</v>
+      </c>
+      <c r="C157" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>70</v>
+      </c>
+      <c r="B158">
+        <v>400</v>
+      </c>
+      <c r="C158" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
         <v>71</v>
       </c>
-      <c r="B157">
+      <c r="B159">
         <v>800</v>
       </c>
-      <c r="C157" t="s">
+      <c r="C159" t="s">
         <v>99</v>
       </c>
     </row>
@@ -3683,7 +3691,7 @@
         <v>39</v>
       </c>
       <c r="B2" s="2">
-        <f>About!B16</f>
+        <f>About!B18</f>
         <v>0.2</v>
       </c>
     </row>
@@ -3692,7 +3700,7 @@
         <v>40</v>
       </c>
       <c r="B3" s="2">
-        <f>About!B17</f>
+        <f>About!B19</f>
         <v>0.6</v>
       </c>
     </row>
@@ -3701,7 +3709,7 @@
         <v>41</v>
       </c>
       <c r="B4" s="2">
-        <f>About!B18</f>
+        <f>About!B20</f>
         <v>3</v>
       </c>
     </row>
@@ -3710,7 +3718,7 @@
         <v>42</v>
       </c>
       <c r="B5" s="2">
-        <f>About!B19</f>
+        <f>About!B21</f>
         <v>0.5</v>
       </c>
     </row>
@@ -3719,7 +3727,7 @@
         <v>38</v>
       </c>
       <c r="B6" s="2">
-        <f>About!B20</f>
+        <f>About!B22</f>
         <v>30000</v>
       </c>
     </row>
@@ -4348,85 +4356,85 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="O8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="P8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="R8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="S8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="T8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="U8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="W8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="X8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Y8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Z8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="AA8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="AB8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">

</xml_diff>